<commit_message>
Update AI microchip sourcing workbook
</commit_message>
<xml_diff>
--- a/public/assets/global-sourcing-ai-microchip-framework.xlsx
+++ b/public/assets/global-sourcing-ai-microchip-framework.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shivenparikh/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shivenparikh/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD2033BA-C111-2E4A-873B-899C5DF6BCD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" activeTab="4" xr2:uid="{9FACD669-EFB5-B74C-B078-C631BE52E6FB}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16840" activeTab="1" xr2:uid="{9FACD669-EFB5-B74C-B078-C631BE52E6FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="Scenario Analysis" sheetId="5" r:id="rId5"/>
     <sheet name="Risk Matrix" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -723,7 +723,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -737,7 +737,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -771,10 +770,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1137,66 +1133,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25" t="s">
+      <c r="B1" s="23" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="23" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="23" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="24" t="s">
+      <c r="A4" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="25" t="s">
+      <c r="B4" s="23" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="23" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="23" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="24" t="s">
+      <c r="A7" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="26" t="s">
+      <c r="B7" s="24" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="24" t="s">
+      <c r="A8" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="23" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1527,27 +1523,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="7" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="8" t="s">
         <v>64</v>
       </c>
       <c r="B2" t="s">
@@ -1567,7 +1563,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="8" t="s">
         <v>73</v>
       </c>
       <c r="B3" t="s">
@@ -1587,7 +1583,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="8" t="s">
         <v>66</v>
       </c>
       <c r="B4" t="s">
@@ -1607,7 +1603,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="8" t="s">
         <v>67</v>
       </c>
       <c r="B5" t="s">
@@ -1627,7 +1623,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="8" t="s">
         <v>74</v>
       </c>
       <c r="B6" t="s">
@@ -1647,7 +1643,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="8" t="s">
         <v>68</v>
       </c>
       <c r="B7" t="s">
@@ -1667,7 +1663,7 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="8" t="s">
         <v>69</v>
       </c>
       <c r="B8" t="s">
@@ -1696,14 +1692,10 @@
   <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="10.83203125" style="5"/>
-    <col min="4" max="4" width="16.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="10.83203125" style="5"/>
-    <col min="8" max="8" width="12.6640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="10.83203125" style="5"/>
-    <col min="12" max="12" width="13.83203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="10.83203125" style="5"/>
+    <col min="1" max="1" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
@@ -1713,7 +1705,7 @@
       <c r="B1" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="6"/>
+      <c r="C1" s="5"/>
       <c r="D1" s="4" t="s">
         <v>63</v>
       </c>
@@ -1746,199 +1738,199 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="B2" s="7">
+      <c r="B2" s="6">
         <v>0.2</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6" t="s">
+      <c r="C2" s="5"/>
+      <c r="D2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="6">
+      <c r="E2" s="5">
         <v>2</v>
       </c>
-      <c r="F2" s="5">
-        <v>3</v>
-      </c>
-      <c r="G2" s="6">
+      <c r="F2">
+        <v>3</v>
+      </c>
+      <c r="G2" s="5">
         <v>4</v>
       </c>
-      <c r="H2" s="6">
-        <v>3</v>
-      </c>
-      <c r="I2" s="6">
+      <c r="H2" s="5">
+        <v>3</v>
+      </c>
+      <c r="I2" s="5">
         <v>2</v>
       </c>
-      <c r="J2" s="6">
-        <v>5</v>
-      </c>
-      <c r="K2" s="6">
+      <c r="J2" s="5">
+        <v>5</v>
+      </c>
+      <c r="K2" s="5">
         <v>1</v>
       </c>
       <c r="L2">
         <f>E2*$B$2+F2*$B$3+G2*$B$4+H2*$B$5+I2*$B$6+J2*$B$7+K2*$B$8</f>
         <v>2.8000000000000003</v>
       </c>
-      <c r="M2" s="5">
+      <c r="M2">
         <f>_xlfn.RANK.EQ(L2,$L$2:$L$4,0)</f>
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="6">
         <v>0.15</v>
       </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6" t="s">
+      <c r="C3" s="5"/>
+      <c r="D3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="6">
-        <v>3</v>
-      </c>
-      <c r="F3" s="5">
-        <v>3</v>
-      </c>
-      <c r="G3" s="6">
+      <c r="E3" s="5">
+        <v>3</v>
+      </c>
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3" s="5">
         <v>4</v>
       </c>
-      <c r="H3" s="6">
-        <v>3</v>
-      </c>
-      <c r="I3" s="6">
-        <v>3</v>
-      </c>
-      <c r="J3" s="6">
-        <v>5</v>
-      </c>
-      <c r="K3" s="6">
+      <c r="H3" s="5">
+        <v>3</v>
+      </c>
+      <c r="I3" s="5">
+        <v>3</v>
+      </c>
+      <c r="J3" s="5">
+        <v>5</v>
+      </c>
+      <c r="K3" s="5">
         <v>2</v>
       </c>
       <c r="L3">
         <f t="shared" ref="L3:L4" si="0">E3*$B$2+F3*$B$3+G3*$B$4+H3*$B$5+I3*$B$6+J3*$B$7+K3*$B$8</f>
         <v>3.3000000000000007</v>
       </c>
-      <c r="M3" s="5">
+      <c r="M3">
         <f t="shared" ref="M3:M4" si="1">_xlfn.RANK.EQ(L3,$L$2:$L$4,0)</f>
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="6">
         <v>0.1</v>
       </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6" t="s">
+      <c r="C4" s="5"/>
+      <c r="D4" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="E4" s="6">
-        <v>5</v>
-      </c>
-      <c r="F4" s="5">
-        <v>5</v>
-      </c>
-      <c r="G4" s="6">
-        <v>5</v>
-      </c>
-      <c r="H4" s="6">
+      <c r="E4" s="5">
+        <v>5</v>
+      </c>
+      <c r="F4">
+        <v>5</v>
+      </c>
+      <c r="G4" s="5">
+        <v>5</v>
+      </c>
+      <c r="H4" s="5">
         <v>4</v>
       </c>
-      <c r="I4" s="6">
-        <v>3</v>
-      </c>
-      <c r="J4" s="6">
-        <v>3</v>
-      </c>
-      <c r="K4" s="6">
+      <c r="I4" s="5">
+        <v>3</v>
+      </c>
+      <c r="J4" s="5">
+        <v>3</v>
+      </c>
+      <c r="K4" s="5">
         <v>4</v>
       </c>
       <c r="L4">
         <f t="shared" si="0"/>
         <v>4.1000000000000005</v>
       </c>
-      <c r="M4" s="5">
+      <c r="M4">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="6">
         <v>0.1</v>
       </c>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="6">
         <v>0.2</v>
       </c>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="6">
         <v>0.15</v>
       </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="6">
         <v>0.1</v>
       </c>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
+      <c r="A11" s="5"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A12" s="6"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
+      <c r="A12" s="5"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1999,672 +1991,672 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="9" t="s">
         <v>123</v>
       </c>
       <c r="B2" s="2"/>
-      <c r="C2" s="11">
+      <c r="C2" s="10">
         <v>0.2</v>
       </c>
-      <c r="D2" s="11">
+      <c r="D2" s="10">
         <v>0.15</v>
       </c>
-      <c r="E2" s="11">
+      <c r="E2" s="10">
         <v>0.1</v>
       </c>
-      <c r="F2" s="11">
+      <c r="F2" s="10">
         <v>0.1</v>
       </c>
-      <c r="G2" s="11">
+      <c r="G2" s="10">
         <v>0.2</v>
       </c>
-      <c r="H2" s="11">
+      <c r="H2" s="10">
         <v>0.15</v>
       </c>
-      <c r="I2" s="11">
+      <c r="I2" s="10">
         <v>0.1</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="9" t="s">
         <v>124</v>
       </c>
       <c r="B3" s="2"/>
-      <c r="C3" s="11">
+      <c r="C3" s="10">
         <v>0.35</v>
       </c>
-      <c r="D3" s="11">
+      <c r="D3" s="10">
         <v>0.15</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="10">
         <v>0.1</v>
       </c>
-      <c r="F3" s="11">
+      <c r="F3" s="10">
         <v>0.05</v>
       </c>
-      <c r="G3" s="11">
+      <c r="G3" s="10">
         <v>0.15</v>
       </c>
-      <c r="H3" s="11">
+      <c r="H3" s="10">
         <v>0.1</v>
       </c>
-      <c r="I3" s="11">
+      <c r="I3" s="10">
         <v>0.1</v>
       </c>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="9" t="s">
         <v>125</v>
       </c>
       <c r="B4" s="2"/>
-      <c r="C4" s="11">
+      <c r="C4" s="10">
         <v>0.15</v>
       </c>
-      <c r="D4" s="11">
+      <c r="D4" s="10">
         <v>0.2</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="10">
         <v>0.05</v>
       </c>
-      <c r="F4" s="11">
+      <c r="F4" s="10">
         <v>0.1</v>
       </c>
-      <c r="G4" s="11">
+      <c r="G4" s="10">
         <v>0.35</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="10">
         <v>0.1</v>
       </c>
-      <c r="I4" s="11">
+      <c r="I4" s="10">
         <v>0.05</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="9" t="s">
         <v>126</v>
       </c>
       <c r="B5" s="2"/>
-      <c r="C5" s="11">
+      <c r="C5" s="10">
         <v>0.25</v>
       </c>
-      <c r="D5" s="11">
+      <c r="D5" s="10">
         <v>0.2</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="10">
         <v>0.1</v>
       </c>
-      <c r="F5" s="11">
+      <c r="F5" s="10">
         <v>0.1</v>
       </c>
-      <c r="G5" s="11">
+      <c r="G5" s="10">
         <v>0.15</v>
       </c>
-      <c r="H5" s="11">
+      <c r="H5" s="10">
         <v>0.1</v>
       </c>
-      <c r="I5" s="11">
+      <c r="I5" s="10">
         <v>0.1</v>
       </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="9" t="s">
         <v>127</v>
       </c>
       <c r="B6" s="2"/>
-      <c r="C6" s="11">
+      <c r="C6" s="10">
         <v>0.15</v>
       </c>
-      <c r="D6" s="11">
+      <c r="D6" s="10">
         <v>0.1</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="10">
         <v>0.25</v>
       </c>
-      <c r="F6" s="11">
+      <c r="F6" s="10">
         <v>0.1</v>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="10">
         <v>0.2</v>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="10">
         <v>0.1</v>
       </c>
-      <c r="I6" s="11">
+      <c r="I6" s="10">
         <v>0.1</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="13">
+      <c r="C7" s="12">
         <v>2</v>
       </c>
-      <c r="D7" s="13">
-        <v>3</v>
-      </c>
-      <c r="E7" s="13">
+      <c r="D7" s="12">
+        <v>3</v>
+      </c>
+      <c r="E7" s="12">
         <v>4</v>
       </c>
-      <c r="F7" s="13">
-        <v>3</v>
-      </c>
-      <c r="G7" s="13">
+      <c r="F7" s="12">
+        <v>3</v>
+      </c>
+      <c r="G7" s="12">
         <v>2</v>
       </c>
-      <c r="H7" s="13">
-        <v>5</v>
-      </c>
-      <c r="I7" s="13">
+      <c r="H7" s="12">
+        <v>5</v>
+      </c>
+      <c r="I7" s="12">
         <v>1</v>
       </c>
-      <c r="J7" s="14">
+      <c r="J7" s="13">
         <v>2.8</v>
       </c>
-      <c r="K7" s="15">
+      <c r="K7" s="14">
         <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="17">
-        <v>3</v>
-      </c>
-      <c r="D8" s="17">
-        <v>3</v>
-      </c>
-      <c r="E8" s="17">
+      <c r="C8" s="9">
+        <v>3</v>
+      </c>
+      <c r="D8" s="9">
+        <v>3</v>
+      </c>
+      <c r="E8" s="9">
         <v>4</v>
       </c>
-      <c r="F8" s="17">
-        <v>3</v>
-      </c>
-      <c r="G8" s="17">
-        <v>3</v>
-      </c>
-      <c r="H8" s="17">
-        <v>5</v>
-      </c>
-      <c r="I8" s="17">
+      <c r="F8" s="9">
+        <v>3</v>
+      </c>
+      <c r="G8" s="9">
+        <v>3</v>
+      </c>
+      <c r="H8" s="9">
+        <v>5</v>
+      </c>
+      <c r="I8" s="9">
         <v>2</v>
       </c>
-      <c r="J8" s="18">
+      <c r="J8" s="16">
         <v>3.3</v>
       </c>
-      <c r="K8" s="19">
+      <c r="K8" s="17">
         <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="20" t="s">
+      <c r="A9" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="C9" s="21">
-        <v>5</v>
-      </c>
-      <c r="D9" s="21">
-        <v>5</v>
-      </c>
-      <c r="E9" s="21">
-        <v>5</v>
-      </c>
-      <c r="F9" s="21">
+      <c r="C9" s="19">
+        <v>5</v>
+      </c>
+      <c r="D9" s="19">
+        <v>5</v>
+      </c>
+      <c r="E9" s="19">
+        <v>5</v>
+      </c>
+      <c r="F9" s="19">
         <v>4</v>
       </c>
-      <c r="G9" s="21">
-        <v>3</v>
-      </c>
-      <c r="H9" s="21">
-        <v>3</v>
-      </c>
-      <c r="I9" s="21">
+      <c r="G9" s="19">
+        <v>3</v>
+      </c>
+      <c r="H9" s="19">
+        <v>3</v>
+      </c>
+      <c r="I9" s="19">
         <v>4</v>
       </c>
-      <c r="J9" s="22">
+      <c r="J9" s="20">
         <v>4.0999999999999996</v>
       </c>
-      <c r="K9" s="23">
+      <c r="K9" s="21">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="12">
         <v>2</v>
       </c>
-      <c r="D10" s="13">
-        <v>3</v>
-      </c>
-      <c r="E10" s="13">
+      <c r="D10" s="12">
+        <v>3</v>
+      </c>
+      <c r="E10" s="12">
         <v>4</v>
       </c>
-      <c r="F10" s="13">
-        <v>3</v>
-      </c>
-      <c r="G10" s="13">
+      <c r="F10" s="12">
+        <v>3</v>
+      </c>
+      <c r="G10" s="12">
         <v>2</v>
       </c>
-      <c r="H10" s="13">
-        <v>5</v>
-      </c>
-      <c r="I10" s="13">
+      <c r="H10" s="12">
+        <v>5</v>
+      </c>
+      <c r="I10" s="12">
         <v>1</v>
       </c>
-      <c r="J10" s="14">
+      <c r="J10" s="13">
         <v>2.6</v>
       </c>
-      <c r="K10" s="15">
+      <c r="K10" s="14">
         <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="17">
-        <v>3</v>
-      </c>
-      <c r="D11" s="17">
-        <v>3</v>
-      </c>
-      <c r="E11" s="17">
+      <c r="C11" s="9">
+        <v>3</v>
+      </c>
+      <c r="D11" s="9">
+        <v>3</v>
+      </c>
+      <c r="E11" s="9">
         <v>4</v>
       </c>
-      <c r="F11" s="17">
-        <v>3</v>
-      </c>
-      <c r="G11" s="17">
-        <v>3</v>
-      </c>
-      <c r="H11" s="17">
-        <v>5</v>
-      </c>
-      <c r="I11" s="17">
+      <c r="F11" s="9">
+        <v>3</v>
+      </c>
+      <c r="G11" s="9">
+        <v>3</v>
+      </c>
+      <c r="H11" s="9">
+        <v>5</v>
+      </c>
+      <c r="I11" s="9">
         <v>2</v>
       </c>
-      <c r="J11" s="18">
+      <c r="J11" s="16">
         <v>3.2</v>
       </c>
-      <c r="K11" s="19">
+      <c r="K11" s="17">
         <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" s="20" t="s">
+      <c r="A12" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="C12" s="21">
-        <v>5</v>
-      </c>
-      <c r="D12" s="21">
-        <v>5</v>
-      </c>
-      <c r="E12" s="21">
-        <v>5</v>
-      </c>
-      <c r="F12" s="21">
+      <c r="C12" s="19">
+        <v>5</v>
+      </c>
+      <c r="D12" s="19">
+        <v>5</v>
+      </c>
+      <c r="E12" s="19">
+        <v>5</v>
+      </c>
+      <c r="F12" s="19">
         <v>4</v>
       </c>
-      <c r="G12" s="21">
-        <v>3</v>
-      </c>
-      <c r="H12" s="21">
-        <v>3</v>
-      </c>
-      <c r="I12" s="21">
+      <c r="G12" s="19">
+        <v>3</v>
+      </c>
+      <c r="H12" s="19">
+        <v>3</v>
+      </c>
+      <c r="I12" s="19">
         <v>4</v>
       </c>
-      <c r="J12" s="22">
+      <c r="J12" s="20">
         <v>4.3499999999999996</v>
       </c>
-      <c r="K12" s="23">
+      <c r="K12" s="21">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="13">
+      <c r="C13" s="12">
         <v>2</v>
       </c>
-      <c r="D13" s="13">
-        <v>3</v>
-      </c>
-      <c r="E13" s="13">
+      <c r="D13" s="12">
+        <v>3</v>
+      </c>
+      <c r="E13" s="12">
         <v>4</v>
       </c>
-      <c r="F13" s="13">
-        <v>3</v>
-      </c>
-      <c r="G13" s="13">
+      <c r="F13" s="12">
+        <v>3</v>
+      </c>
+      <c r="G13" s="12">
         <v>2</v>
       </c>
-      <c r="H13" s="13">
-        <v>5</v>
-      </c>
-      <c r="I13" s="13">
+      <c r="H13" s="12">
+        <v>5</v>
+      </c>
+      <c r="I13" s="12">
         <v>1</v>
       </c>
-      <c r="J13" s="14">
+      <c r="J13" s="13">
         <v>2.65</v>
       </c>
-      <c r="K13" s="15">
+      <c r="K13" s="14">
         <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="17">
-        <v>3</v>
-      </c>
-      <c r="D14" s="17">
-        <v>3</v>
-      </c>
-      <c r="E14" s="17">
+      <c r="C14" s="9">
+        <v>3</v>
+      </c>
+      <c r="D14" s="9">
+        <v>3</v>
+      </c>
+      <c r="E14" s="9">
         <v>4</v>
       </c>
-      <c r="F14" s="17">
-        <v>3</v>
-      </c>
-      <c r="G14" s="17">
-        <v>3</v>
-      </c>
-      <c r="H14" s="17">
-        <v>5</v>
-      </c>
-      <c r="I14" s="17">
+      <c r="F14" s="9">
+        <v>3</v>
+      </c>
+      <c r="G14" s="9">
+        <v>3</v>
+      </c>
+      <c r="H14" s="9">
+        <v>5</v>
+      </c>
+      <c r="I14" s="9">
         <v>2</v>
       </c>
-      <c r="J14" s="18">
+      <c r="J14" s="16">
         <v>3.2</v>
       </c>
-      <c r="K14" s="19">
+      <c r="K14" s="17">
         <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" s="20" t="s">
+      <c r="A15" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="B15" s="21" t="s">
+      <c r="B15" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="C15" s="21">
-        <v>5</v>
-      </c>
-      <c r="D15" s="21">
-        <v>5</v>
-      </c>
-      <c r="E15" s="21">
-        <v>5</v>
-      </c>
-      <c r="F15" s="21">
+      <c r="C15" s="19">
+        <v>5</v>
+      </c>
+      <c r="D15" s="19">
+        <v>5</v>
+      </c>
+      <c r="E15" s="19">
+        <v>5</v>
+      </c>
+      <c r="F15" s="19">
         <v>4</v>
       </c>
-      <c r="G15" s="21">
-        <v>3</v>
-      </c>
-      <c r="H15" s="21">
-        <v>3</v>
-      </c>
-      <c r="I15" s="21">
+      <c r="G15" s="19">
+        <v>3</v>
+      </c>
+      <c r="H15" s="19">
+        <v>3</v>
+      </c>
+      <c r="I15" s="19">
         <v>4</v>
       </c>
-      <c r="J15" s="22">
+      <c r="J15" s="20">
         <v>3.95</v>
       </c>
-      <c r="K15" s="23">
+      <c r="K15" s="21">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B16" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="13">
+      <c r="C16" s="12">
         <v>2</v>
       </c>
-      <c r="D16" s="13">
-        <v>3</v>
-      </c>
-      <c r="E16" s="13">
+      <c r="D16" s="12">
+        <v>3</v>
+      </c>
+      <c r="E16" s="12">
         <v>4</v>
       </c>
-      <c r="F16" s="13">
-        <v>3</v>
-      </c>
-      <c r="G16" s="13">
+      <c r="F16" s="12">
+        <v>3</v>
+      </c>
+      <c r="G16" s="12">
         <v>2</v>
       </c>
-      <c r="H16" s="13">
-        <v>5</v>
-      </c>
-      <c r="I16" s="13">
+      <c r="H16" s="12">
+        <v>5</v>
+      </c>
+      <c r="I16" s="12">
         <v>1</v>
       </c>
-      <c r="J16" s="14">
+      <c r="J16" s="13">
         <v>2.7</v>
       </c>
-      <c r="K16" s="15">
+      <c r="K16" s="14">
         <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A17" s="16" t="s">
+      <c r="A17" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="17">
-        <v>3</v>
-      </c>
-      <c r="D17" s="17">
-        <v>3</v>
-      </c>
-      <c r="E17" s="17">
+      <c r="C17" s="9">
+        <v>3</v>
+      </c>
+      <c r="D17" s="9">
+        <v>3</v>
+      </c>
+      <c r="E17" s="9">
         <v>4</v>
       </c>
-      <c r="F17" s="17">
-        <v>3</v>
-      </c>
-      <c r="G17" s="17">
-        <v>3</v>
-      </c>
-      <c r="H17" s="17">
-        <v>5</v>
-      </c>
-      <c r="I17" s="17">
+      <c r="F17" s="9">
+        <v>3</v>
+      </c>
+      <c r="G17" s="9">
+        <v>3</v>
+      </c>
+      <c r="H17" s="9">
+        <v>5</v>
+      </c>
+      <c r="I17" s="9">
         <v>2</v>
       </c>
-      <c r="J17" s="18">
+      <c r="J17" s="16">
         <v>3.2</v>
       </c>
-      <c r="K17" s="19">
+      <c r="K17" s="17">
         <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="20" t="s">
+      <c r="A18" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="B18" s="21" t="s">
+      <c r="B18" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="C18" s="21">
-        <v>5</v>
-      </c>
-      <c r="D18" s="21">
-        <v>5</v>
-      </c>
-      <c r="E18" s="21">
-        <v>5</v>
-      </c>
-      <c r="F18" s="21">
+      <c r="C18" s="19">
+        <v>5</v>
+      </c>
+      <c r="D18" s="19">
+        <v>5</v>
+      </c>
+      <c r="E18" s="19">
+        <v>5</v>
+      </c>
+      <c r="F18" s="19">
         <v>4</v>
       </c>
-      <c r="G18" s="21">
-        <v>3</v>
-      </c>
-      <c r="H18" s="21">
-        <v>3</v>
-      </c>
-      <c r="I18" s="21">
+      <c r="G18" s="19">
+        <v>3</v>
+      </c>
+      <c r="H18" s="19">
+        <v>3</v>
+      </c>
+      <c r="I18" s="19">
         <v>4</v>
       </c>
-      <c r="J18" s="22">
+      <c r="J18" s="20">
         <v>4.3</v>
       </c>
-      <c r="K18" s="23">
+      <c r="K18" s="21">
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="B19" s="13" t="s">
+      <c r="B19" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C19" s="13">
+      <c r="C19" s="12">
         <v>2</v>
       </c>
-      <c r="D19" s="13">
-        <v>3</v>
-      </c>
-      <c r="E19" s="13">
+      <c r="D19" s="12">
+        <v>3</v>
+      </c>
+      <c r="E19" s="12">
         <v>4</v>
       </c>
-      <c r="F19" s="13">
-        <v>3</v>
-      </c>
-      <c r="G19" s="13">
+      <c r="F19" s="12">
+        <v>3</v>
+      </c>
+      <c r="G19" s="12">
         <v>2</v>
       </c>
-      <c r="H19" s="13">
-        <v>5</v>
-      </c>
-      <c r="I19" s="13">
+      <c r="H19" s="12">
+        <v>5</v>
+      </c>
+      <c r="I19" s="12">
         <v>1</v>
       </c>
-      <c r="J19" s="14">
+      <c r="J19" s="13">
         <v>2.9</v>
       </c>
-      <c r="K19" s="15">
+      <c r="K19" s="14">
         <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A20" s="16" t="s">
+      <c r="A20" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C20" s="17">
-        <v>3</v>
-      </c>
-      <c r="D20" s="17">
-        <v>3</v>
-      </c>
-      <c r="E20" s="17">
+      <c r="C20" s="9">
+        <v>3</v>
+      </c>
+      <c r="D20" s="9">
+        <v>3</v>
+      </c>
+      <c r="E20" s="9">
         <v>4</v>
       </c>
-      <c r="F20" s="17">
-        <v>3</v>
-      </c>
-      <c r="G20" s="17">
-        <v>3</v>
-      </c>
-      <c r="H20" s="17">
-        <v>5</v>
-      </c>
-      <c r="I20" s="17">
+      <c r="F20" s="9">
+        <v>3</v>
+      </c>
+      <c r="G20" s="9">
+        <v>3</v>
+      </c>
+      <c r="H20" s="9">
+        <v>5</v>
+      </c>
+      <c r="I20" s="9">
         <v>2</v>
       </c>
-      <c r="J20" s="18">
+      <c r="J20" s="16">
         <v>3.35</v>
       </c>
-      <c r="K20" s="19">
+      <c r="K20" s="17">
         <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A21" s="20" t="s">
+      <c r="A21" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="B21" s="21" t="s">
+      <c r="B21" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="C21" s="21">
-        <v>5</v>
-      </c>
-      <c r="D21" s="21">
-        <v>5</v>
-      </c>
-      <c r="E21" s="21">
-        <v>5</v>
-      </c>
-      <c r="F21" s="21">
+      <c r="C21" s="19">
+        <v>5</v>
+      </c>
+      <c r="D21" s="19">
+        <v>5</v>
+      </c>
+      <c r="E21" s="19">
+        <v>5</v>
+      </c>
+      <c r="F21" s="19">
         <v>4</v>
       </c>
-      <c r="G21" s="21">
-        <v>3</v>
-      </c>
-      <c r="H21" s="21">
-        <v>3</v>
-      </c>
-      <c r="I21" s="21">
+      <c r="G21" s="19">
+        <v>3</v>
+      </c>
+      <c r="H21" s="19">
+        <v>3</v>
+      </c>
+      <c r="I21" s="19">
         <v>4</v>
       </c>
-      <c r="J21" s="22">
+      <c r="J21" s="20">
         <v>4.2</v>
       </c>
-      <c r="K21" s="23">
+      <c r="K21" s="21">
         <v>1</v>
       </c>
     </row>

</xml_diff>